<commit_message>
resolution of the Data Acquisition Phase
</commit_message>
<xml_diff>
--- a/final_sample_sheet.xlsx
+++ b/final_sample_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbolden/Desktop/SMR2026/BIDS26_Project3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520ECB95-47FB-A841-AC01-369122556E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62347B1A-77D2-944D-AE2F-809C921AB746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="960" windowWidth="16880" windowHeight="21040" xr2:uid="{DFF43703-4A32-3544-8BA4-F4F8ABE3CD82}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>Citation</t>
   </si>
@@ -47,12 +47,6 @@
     <t>Conditions</t>
   </si>
   <si>
-    <t>Reported Cell Cnt (post QC)</t>
-  </si>
-  <si>
-    <t>Cell Cnt after Read in</t>
-  </si>
-  <si>
     <t>Lib Prep Protrocol</t>
   </si>
   <si>
@@ -266,10 +260,55 @@
     <t>Chromium Single Cell 5'</t>
   </si>
   <si>
-    <t>Chromium  and Slide-Seq (only SC samples used)</t>
-  </si>
-  <si>
     <t>Available</t>
+  </si>
+  <si>
+    <t>Cell Cnt after Read in (preQC)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>36000(preQC).5288 (postQC)</t>
+  </si>
+  <si>
+    <t>~21,000 (postQC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author Reported Cell Cnt </t>
+  </si>
+  <si>
+    <t>36424(preQC)</t>
+  </si>
+  <si>
+    <t>* only read in the human tumor samples</t>
+  </si>
+  <si>
+    <t>Chromium   (only SC samples used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* only read in 5 Healthy samples and 10 paired Adj.N and Tumor core samples due to lack computational storage </t>
+  </si>
+  <si>
+    <t>91,498*</t>
+  </si>
+  <si>
+    <t>6,730*</t>
+  </si>
+  <si>
+    <t>Total Cell Cnt (PreQC): 187,652</t>
+  </si>
+  <si>
+    <t>Healthy Samples: 5</t>
+  </si>
+  <si>
+    <t>tumor_core:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tumor Only: </t>
+  </si>
+  <si>
+    <t>Adj_Normal:</t>
   </si>
 </sst>
 </file>
@@ -396,7 +435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -417,6 +456,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -753,10 +798,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFFBF3AE-6674-994A-9C3A-3B613D678BB9}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="52" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="52" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -768,89 +813,107 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="69" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="69" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="8">
+        <v>36424</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="69" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="s">
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="8">
+        <v>53000</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="69" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
+      <c r="H4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="52" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="52" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
@@ -858,26 +921,58 @@
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" ht="103" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="239" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="E6" s="8">
+        <v>179359</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F14" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
At integration taking a short break
</commit_message>
<xml_diff>
--- a/final_sample_sheet.xlsx
+++ b/final_sample_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbolden/Desktop/SMR2026/BIDS26_Project3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC94437-4A27-8F41-A8C9-1E5A149A72CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0724ABF-C741-9C42-930D-9AAE8B19EEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15600" yWindow="940" windowWidth="18460" windowHeight="21060" xr2:uid="{DFF43703-4A32-3544-8BA4-F4F8ABE3CD82}"/>
+    <workbookView xWindow="15580" yWindow="940" windowWidth="18460" windowHeight="21060" xr2:uid="{DFF43703-4A32-3544-8BA4-F4F8ABE3CD82}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -275,9 +275,6 @@
     <t>There was no need to perform manual thresholds. Authors distributed clean dataset</t>
   </si>
   <si>
-    <t>Total  Cel Cnt (PostQC): 143,582</t>
-  </si>
-  <si>
     <t>Human only Cells and Samples</t>
   </si>
   <si>
@@ -318,6 +315,9 @@
   </si>
   <si>
     <t xml:space="preserve">This Balance needs to change I suggest that we take away the benign cells completely and at least 5 more healthy samples	</t>
+  </si>
+  <si>
+    <t>Total  Cel Cnt (PostQC): 143,851</t>
   </si>
 </sst>
 </file>
@@ -480,18 +480,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -505,11 +493,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -850,36 +850,36 @@
   <sheetData>
     <row r="1" spans="1:10" ht="69" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="86" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2"/>
@@ -907,7 +907,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="154" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -939,31 +939,31 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="51" x14ac:dyDescent="0.2">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="13" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="13" t="s">
         <v>21</v>
       </c>
       <c r="J4" t="s">
@@ -971,23 +971,23 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="154" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="7"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
       <c r="J5" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="205" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -1020,103 +1020,103 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E11" s="6" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F9" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F10" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E11" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>47</v>
+      <c r="F11" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="H11">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E12" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>48</v>
+      <c r="E12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="H12">
         <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E13" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>49</v>
+      <c r="E13" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>48</v>
       </c>
       <c r="H13">
         <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>50</v>
+      <c r="F14" s="7" t="s">
+        <v>49</v>
       </c>
       <c r="H14">
         <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E15" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>51</v>
+      <c r="E15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>50</v>
       </c>
       <c r="H15">
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E16" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>52</v>
+      <c r="E16" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="H16">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E17" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13">
+      <c r="E17" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9">
         <f>SUM(H11:H16)</f>
         <v>76</v>
       </c>
     </row>
     <row r="19" spans="5:8" x14ac:dyDescent="0.2">
-      <c r="E19" s="10" t="s">
-        <v>54</v>
+      <c r="E19" s="6" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>